<commit_message>
Update planning document and feature board
Co-authored-by: Hafidz Arifin <hafidz.harifin@gmail.com>
Signed-off-by: SirGankalot <73303677+SirGankalot@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/Deliverables/sprint-14/planning-documents.xlsx
+++ b/Deliverables/sprint-14/planning-documents.xlsx
@@ -816,16 +816,16 @@
     <t>Create Demo Day Presenation</t>
   </si>
   <si>
-    <t>Create Project Report</t>
-  </si>
-  <si>
-    <t>Tasks related to Industry Partner</t>
-  </si>
-  <si>
-    <t>Merging the code with main repo of partner</t>
-  </si>
-  <si>
-    <t>Final Bug Fixes</t>
+    <t>Merge Project to Core Repository based on Shell Feedback</t>
+  </si>
+  <si>
+    <t>Project Report</t>
+  </si>
+  <si>
+    <t>Preparing and showcasing Implementation on Demo Day</t>
+  </si>
+  <si>
+    <t>Finalize user, (technical) design, and build/deploy documentation</t>
   </si>
   <si>
     <t>Feature Definition of Done</t>
@@ -2330,11 +2330,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1368015913"/>
-        <c:axId val="538100882"/>
+        <c:axId val="1528455627"/>
+        <c:axId val="1778033680"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1368015913"/>
+        <c:axId val="1528455627"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2386,10 +2386,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="538100882"/>
+        <c:crossAx val="1778033680"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="538100882"/>
+        <c:axId val="1778033680"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2464,7 +2464,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1368015913"/>
+        <c:crossAx val="1528455627"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2553,11 +2553,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="676667670"/>
-        <c:axId val="1125422979"/>
+        <c:axId val="1831747731"/>
+        <c:axId val="1619044227"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="676667670"/>
+        <c:axId val="1831747731"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2609,10 +2609,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1125422979"/>
+        <c:crossAx val="1619044227"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="1125422979"/>
+        <c:axId val="1619044227"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2687,7 +2687,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="676667670"/>
+        <c:crossAx val="1831747731"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -2776,11 +2776,11 @@
             </c:numRef>
           </c:val>
         </c:ser>
-        <c:axId val="1035545035"/>
-        <c:axId val="718679777"/>
+        <c:axId val="660865656"/>
+        <c:axId val="274882298"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="1035545035"/>
+        <c:axId val="660865656"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2832,10 +2832,10 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="718679777"/>
+        <c:crossAx val="274882298"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="718679777"/>
+        <c:axId val="274882298"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2910,7 +2910,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="1035545035"/>
+        <c:crossAx val="660865656"/>
       </c:valAx>
     </c:plotArea>
     <c:legend>
@@ -5073,11 +5073,11 @@
       <c r="C5" s="80"/>
       <c r="D5" s="81">
         <f>SUM(D9:D16)</f>
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="E5" s="81">
         <f>D5</f>
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="F5" s="80"/>
       <c r="G5" s="80"/>
@@ -5128,7 +5128,7 @@
       </c>
       <c r="E9" s="81">
         <f>$D$5 - D9</f>
-        <v>103</v>
+        <v>99</v>
       </c>
       <c r="F9" s="81">
         <f>SUM(F21:F27)</f>
@@ -5136,7 +5136,7 @@
       </c>
       <c r="G9" s="81">
         <f>$D$5-F9</f>
-        <v>102</v>
+        <v>98</v>
       </c>
     </row>
     <row r="10">
@@ -5153,7 +5153,7 @@
       </c>
       <c r="E10" s="87">
         <f t="shared" ref="E10:E16" si="2">E9-D10</f>
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="F10" s="87">
         <f>SUM(F28:F34)</f>
@@ -5161,7 +5161,7 @@
       </c>
       <c r="G10" s="87">
         <f t="shared" ref="G10:G16" si="3">G9-F10</f>
-        <v>89</v>
+        <v>85</v>
       </c>
     </row>
     <row r="11">
@@ -5179,7 +5179,7 @@
       </c>
       <c r="E11" s="81">
         <f t="shared" si="2"/>
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="F11" s="81">
         <f>SUM(F35:F41)</f>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="G11" s="81">
         <f t="shared" si="3"/>
-        <v>75</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12">
@@ -5205,7 +5205,7 @@
       </c>
       <c r="E12" s="87">
         <f t="shared" si="2"/>
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="F12" s="87">
         <f>SUM(F42:F49)</f>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="G12" s="87">
         <f t="shared" si="3"/>
-        <v>60</v>
+        <v>56</v>
       </c>
     </row>
     <row r="13">
@@ -5231,7 +5231,7 @@
       </c>
       <c r="E13" s="81">
         <f t="shared" si="2"/>
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="F13" s="81">
         <f>SUM(F50:F56)</f>
@@ -5239,7 +5239,7 @@
       </c>
       <c r="G13" s="81">
         <f t="shared" si="3"/>
-        <v>48</v>
+        <v>44</v>
       </c>
     </row>
     <row r="14">
@@ -5257,7 +5257,7 @@
       </c>
       <c r="E14" s="87">
         <f t="shared" si="2"/>
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F14" s="87">
         <f>SUM(F57:F63)</f>
@@ -5265,7 +5265,7 @@
       </c>
       <c r="G14" s="87">
         <f t="shared" si="3"/>
-        <v>38</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15">
@@ -5283,7 +5283,7 @@
       </c>
       <c r="E15" s="81">
         <f t="shared" si="2"/>
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="F15" s="81">
         <f>SUM(F64:F70)</f>
@@ -5291,7 +5291,7 @@
       </c>
       <c r="G15" s="81">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>18</v>
       </c>
     </row>
     <row r="16">
@@ -5305,7 +5305,7 @@
       <c r="C16" s="74"/>
       <c r="D16" s="87">
         <f>SUM(D71:D78)</f>
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="E16" s="87">
         <f t="shared" si="2"/>
@@ -5313,11 +5313,11 @@
       </c>
       <c r="F16" s="87">
         <f>SUM(F71:F78)</f>
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G16" s="87">
         <f t="shared" si="3"/>
-        <v>22</v>
+        <v>11</v>
       </c>
     </row>
     <row r="17">
@@ -6067,7 +6067,9 @@
         <v>3.0</v>
       </c>
       <c r="E72" s="99"/>
-      <c r="F72" s="99"/>
+      <c r="F72" s="89">
+        <v>1.0</v>
+      </c>
       <c r="G72" s="99"/>
     </row>
     <row r="73">
@@ -6077,10 +6079,12 @@
         <v>262</v>
       </c>
       <c r="D73" s="101">
-        <v>5.0</v>
+        <v>1.0</v>
       </c>
       <c r="E73" s="80"/>
-      <c r="F73" s="80"/>
+      <c r="F73" s="97">
+        <v>1.0</v>
+      </c>
       <c r="G73" s="80"/>
     </row>
     <row r="74">
@@ -6093,7 +6097,9 @@
         <v>3.0</v>
       </c>
       <c r="E74" s="99"/>
-      <c r="F74" s="99"/>
+      <c r="F74" s="89">
+        <v>3.0</v>
+      </c>
       <c r="G74" s="99"/>
     </row>
     <row r="75">
@@ -6106,7 +6112,9 @@
         <v>3.0</v>
       </c>
       <c r="E75" s="80"/>
-      <c r="F75" s="80"/>
+      <c r="F75" s="97">
+        <v>2.0</v>
+      </c>
       <c r="G75" s="80"/>
     </row>
     <row r="76">
@@ -9773,7 +9781,7 @@
       </c>
       <c r="B15" s="64">
         <f>'Final Project Release plan'!F16</f>
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="16">

</xml_diff>